<commit_message>
Add Trade_Journal.py - tracks alert-to-exit lifecycle and computes win rate/R-multiple statistics
</commit_message>
<xml_diff>
--- a/RESEARCH_WATCHLIST.xlsx
+++ b/RESEARCH_WATCHLIST.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -618,7 +618,7 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.3283828382838284</v>
+        <v>0.2590460526315789</v>
       </c>
       <c r="R2" t="n">
         <v>0.2962962962962963</v>
@@ -668,7 +668,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -720,7 +720,7 @@
       </c>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="n">
-        <v>0.6443894389438944</v>
+        <v>0.618421052631579</v>
       </c>
       <c r="R3" t="n">
         <v>0.8518518518518519</v>
@@ -770,7 +770,7 @@
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -822,7 +822,7 @@
       </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="n">
-        <v>0.5016501650165016</v>
+        <v>0.4876644736842105</v>
       </c>
       <c r="R4" t="n">
         <v>0.2962962962962963</v>
@@ -872,7 +872,7 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -924,7 +924,7 @@
       </c>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="n">
-        <v>0.6806930693069307</v>
+        <v>0.8889802631578947</v>
       </c>
       <c r="R5" t="n">
         <v>0.9629629629629629</v>
@@ -974,7 +974,7 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="n">
-        <v>0.3275577557755776</v>
+        <v>0.3009868421052632</v>
       </c>
       <c r="R6" t="n">
         <v>0.7407407407407407</v>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1088,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
-        <v>0.1996699669966997</v>
+        <v>0.2639802631578947</v>
       </c>
       <c r="R7" t="n">
         <v>0.7037037037037037</v>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
-        <v>0.2813531353135313</v>
+        <v>0.109375</v>
       </c>
       <c r="R8" t="n">
         <v>0.2962962962962963</v>
@@ -1280,7 +1280,7 @@
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1292,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="n">
-        <v>0.1443894389438944</v>
+        <v>0.1291118421052632</v>
       </c>
       <c r="R9" t="n">
         <v>0.2962962962962963</v>
@@ -1382,7 +1382,7 @@
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1434,7 +1434,7 @@
       </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
-        <v>0.9760726072607261</v>
+        <v>0.740953947368421</v>
       </c>
       <c r="R10" t="n">
         <v>0.8148148148148148</v>
@@ -1484,7 +1484,7 @@
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
-        <v>0.745049504950495</v>
+        <v>0.4934210526315789</v>
       </c>
       <c r="R11" t="n">
         <v>0.6296296296296297</v>
@@ -1586,7 +1586,7 @@
       </c>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1598,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="n">
-        <v>0.5915841584158416</v>
+        <v>0.6019736842105263</v>
       </c>
       <c r="R12" t="n">
         <v>0.9259259259259259</v>
@@ -1688,7 +1688,7 @@
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="n">
-        <v>0.2995049504950495</v>
+        <v>0.3766447368421053</v>
       </c>
       <c r="R13" t="n">
         <v>0.2962962962962963</v>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -1802,7 +1802,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>0.3877887788778878</v>
+        <v>0.3881578947368421</v>
       </c>
       <c r="R14" t="n">
         <v>0.2962962962962963</v>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="AD14" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="n">
-        <v>0.8613861386138614</v>
+        <v>0.9514802631578947</v>
       </c>
       <c r="R15" t="n">
         <v>0.2962962962962963</v>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="AD15" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="n">
-        <v>0.1831683168316832</v>
+        <v>0.3955592105263158</v>
       </c>
       <c r="R16" t="n">
         <v>0.6666666666666666</v>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2148,7 +2148,7 @@
       </c>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="n">
-        <v>0.372937293729373</v>
+        <v>0.3470394736842105</v>
       </c>
       <c r="R17" t="n">
         <v>0.8888888888888888</v>
@@ -2198,7 +2198,7 @@
       </c>
       <c r="AD17" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="n">
-        <v>0.608085808580858</v>
+        <v>0.6167763157894737</v>
       </c>
       <c r="R18" t="n">
         <v>0.2962962962962963</v>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="AD18" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -2312,7 +2312,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="n">
-        <v>0.3077557755775577</v>
+        <v>0.2368421052631579</v>
       </c>
       <c r="R19" t="n">
         <v>0.5925925925925926</v>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="AD19" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2454,7 +2454,7 @@
       </c>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="n">
-        <v>0.6526402640264026</v>
+        <v>0.8930921052631579</v>
       </c>
       <c r="R20" t="n">
         <v>0.2962962962962963</v>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="AD20" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -2516,7 +2516,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="n">
-        <v>0.462046204620462</v>
+        <v>0.3774671052631579</v>
       </c>
       <c r="R21" t="n">
         <v>0.2962962962962963</v>
@@ -2606,7 +2606,7 @@
       </c>
       <c r="AD21" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -2618,7 +2618,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -2658,7 +2658,7 @@
       </c>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="n">
-        <v>0.863036303630363</v>
+        <v>0.8626644736842105</v>
       </c>
       <c r="R22" t="n">
         <v>0.2962962962962963</v>
@@ -2708,7 +2708,7 @@
       </c>
       <c r="AD22" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -2720,7 +2720,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="n">
-        <v>0.1914191419141914</v>
+        <v>0.03042763157894737</v>
       </c>
       <c r="R23" t="n">
         <v>1</v>
@@ -2810,7 +2810,7 @@
       </c>
       <c r="AD23" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="n">
-        <v>0.7054455445544554</v>
+        <v>0.7425986842105263</v>
       </c>
       <c r="R24" t="n">
         <v>0.7777777777777778</v>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="AD24" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -2924,7 +2924,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="n">
-        <v>0.03795379537953796</v>
+        <v>0.03865131578947369</v>
       </c>
       <c r="R25" t="n">
         <v>0.2962962962962963</v>
@@ -3002,7 +3002,7 @@
       </c>
       <c r="AD25" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -3014,7 +3014,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3054,7 +3054,7 @@
       </c>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="n">
-        <v>0.4942244224422442</v>
+        <v>0.6175986842105263</v>
       </c>
       <c r="R26" t="n">
         <v>0.2962962962962963</v>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="AD26" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -3104,7 +3104,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3144,7 +3144,7 @@
       </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="n">
-        <v>0.8358085808580858</v>
+        <v>0.8125</v>
       </c>
       <c r="R27" t="n">
         <v>0.2962962962962963</v>
@@ -3182,7 +3182,7 @@
       </c>
       <c r="AD27" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="n">
-        <v>0.9018151815181518</v>
+        <v>0.9111842105263158</v>
       </c>
       <c r="R28" t="n">
         <v>0.2962962962962963</v>
@@ -3272,7 +3272,7 @@
       </c>
       <c r="AD28" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3284,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="AD29" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -3366,7 +3366,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="AD30" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -3518,7 +3518,7 @@
       </c>
       <c r="AD31" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -3530,7 +3530,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="AD32" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -3612,7 +3612,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -3682,7 +3682,7 @@
       </c>
       <c r="AD33" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -3694,7 +3694,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="AD34" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="AD35" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -3928,7 +3928,7 @@
       </c>
       <c r="AD36" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4010,7 +4010,7 @@
       </c>
       <c r="AD37" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -4022,7 +4022,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4092,7 +4092,7 @@
       </c>
       <c r="AD38" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -4174,7 +4174,7 @@
       </c>
       <c r="AD39" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="AD40" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -4268,7 +4268,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -4338,7 +4338,7 @@
       </c>
       <c r="AD41" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>

</xml_diff>